<commit_message>
Add non-blocking GitHub release update check (UpdateCheck.enabled, default on)
UpdateCheck.cs runs a background task (Task.Run, 10s timeout, cached result,
6h re-check throttle from the UDFs) against the GitHub releases API. It never
touches the Excel main thread; failures (offline, rate limit) are silent and
only logged. The result is exposed through RedisUDFUpdateAvailable and
RedisUDFUpdateInfo.

Config: new UpdateCheck section in RedisExcel.json with "enabled" defaulting
to true - backward compatible; sample config files updated. The check starts
from AddIn.AutoOpen.

Also: System.Net.Http reference in the add-in csproj; 14 new unit tests
(version comparison/normalization, config default); Readme UDF table and JSON
sample; AGENTS layout; CHANGELOG v1.1.1 entry. Validated with 40 unit tests,
smoke tests and the Excel end-to-end suite (all pass).
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Trabalho\rs\redisexcel\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1FD7105-75C2-4302-A59D-83DC5EB54AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D21BDBF1-E01C-4D63-B10D-7D4B6F020492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5640" yWindow="-28770" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{B75BC407-9E05-497C-9A85-4480C64E9676}"/>
+    <workbookView xWindow="5640" yWindow="-28770" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{EBB1DE32-8B08-455A-90D2-CBB6CF60AFAB}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -568,7 +568,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D7C84E4-562D-44D2-8FD0-F3F4BDAB2D08}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{648815EF-15FD-4223-A28D-F642C3019C5B}">
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -737,7 +737,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{670B3D57-A4DF-4E4E-8897-19D727618726}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91F829D1-B7A4-4FCC-8120-0BFAF2059B03}">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Simplify update check: boolean config, single TRUE/FALSE UDF, 6h background refresh
Config: "UpdateCheck": true|false is now a plain boolean (default on),
replacing the { "enabled": ... } object introduced in v1.1.1.

Worksheet surface: only RedisUDFUpdateAvailable(), returning TRUE/FALSE (the
RedisUDFUpdateInfo matrix from v1.1.1 is gone). The result is still stored so
the function never blocks Excel; the background check runs at add-in load and
refreshes at most every 6 hours when the function recalculates.

Samples, Readme and CHANGELOG (v1.1.2) updated; 40 unit tests and the Excel
end-to-end suite pass.
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Trabalho\rs\redisexcel\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D21BDBF1-E01C-4D63-B10D-7D4B6F020492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AF803E0-5C49-42B9-9924-E0F868EDFFDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5640" yWindow="-28770" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{EBB1DE32-8B08-455A-90D2-CBB6CF60AFAB}"/>
+    <workbookView xWindow="5640" yWindow="-28770" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{6153C744-F487-4E41-AB5B-2473C7925BE8}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -568,7 +568,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{648815EF-15FD-4223-A28D-F642C3019C5B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33742EAC-9AC9-4E2A-A218-0C9C4BE199D2}">
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -737,7 +737,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91F829D1-B7A4-4FCC-8120-0BFAF2059B03}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2270D1C5-1EC3-4EB8-8294-80B6A0AB7154}">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Cache Redis wrappers, pipeline multi-key UDFs, dedup HGETALL polling
- RedisConnectionManager caches IDatabase and ISubscriber wrappers per
  host/pool (volatile worksheet functions call them constantly and
  ConnectionMultiplexer.GetDatabase()/GetSubscriber() allocate per call);
  caches are cleared on Shutdown. The RedisUDF publish paths use the cached
  subscriber.
- RedisUDFExistsMultiples, RedisUDFTTLMultiples and
  RedisUDFHashGetFieldMultipleKeys now pipeline every key in a single batch
  round trip instead of one synchronous command per key.
- RTD HGETALL polling compares the returned hash field-by-field with the
  previous tick (RedisResultFormatter.HashEquals) and skips unchanged hashes
  before formatting and pushing to Excel (extends SkipRepeatedMessages).
- Smoke tests assert the wrapper caching; unit tests cover HashEquals; the
  E2E workbook now exercises all three pipelined functions.

Validated: 42 unit tests, smoke tests and the Excel end-to-end suite pass.
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Trabalho\rs\redisexcel\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AB7176B-244D-4F21-8680-880582F4DB96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F837E30E-E852-4F1E-9DAF-FA514E05042E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5640" yWindow="-28770" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{0188E7DD-49A3-410D-ABB2-C6BA0600603B}"/>
+    <workbookView xWindow="5640" yWindow="-28770" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{FF395B52-4190-4BF1-AE53-299997F12B4F}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>RedisExcel UDF tests (host localhost:6379, prefix test.redisexcel)</t>
   </si>
@@ -106,6 +106,15 @@
   </si>
   <si>
     <t>ConnectionCount</t>
+  </si>
+  <si>
+    <t>ExistsMultiples</t>
+  </si>
+  <si>
+    <t>TTLMultiples</t>
+  </si>
+  <si>
+    <t>HashGetFieldMultipleKeys</t>
   </si>
   <si>
     <t>RedisExcel RTD tests (host localhost:6379)</t>
@@ -568,8 +577,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E534DB3-4378-4335-A6F9-524FD54A5A47}">
-  <dimension ref="A1:G14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{927A6C7C-9621-4CA0-8B6B-51495E5D03BF}">
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -729,6 +738,42 @@
       <c r="B14">
         <f ca="1">_xll.RedisUDFConnectionCount()</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" t="str">
+        <f ca="1">INDEX(_xll.RedisUDFExistsMultiples({"test.redisexcel.key","test.redisexcel.missing"},"localhost:6379"),1,2)</f>
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" t="str">
+        <f ca="1">INDEX(_xll.RedisUDFTTLMultiples({"test.redisexcel.key"},"localhost:6379"),1,2)</f>
+        <v>-1</v>
+      </c>
+      <c r="C16">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="str">
+        <f ca="1">INDEX(_xll.RedisUDFHashGetFieldMultipleKeys({"test.redisexcel.hash","test.redisexcel.hash"},"campo1","localhost:6379"),2,2)</f>
+        <v>valor1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -737,13 +782,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E32D44C4-38AB-41F3-8D41-0941621B884B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F3DEB0-CC94-4B2A-A945-A35DD515B1E7}">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -759,7 +804,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B4" t="str">
         <f>RTD("redisrtd",,"GET","test.redisexcel.key","localhost:6379")</f>
@@ -771,7 +816,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B5" t="str">
         <f>RTD("redisrtd",,"HGET","test.redisexcel.hash","campo1","localhost:6379")</f>
@@ -783,19 +828,19 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B6" t="str">
         <f>RTD("redisrtd",,"HGETALL","test.redisexcel.hash","localhost:6379")</f>
         <v>{"campo1":"valor1"}</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B7" t="str">
         <f>RTD("redisrtd",,"SUB","test.redisexcel.rtd","localhost:6379")</f>
@@ -804,7 +849,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B8" t="str">
         <f>RTD("redisrtd",,"PSUB","test.redisexcel.rtd*","localhost:6379")</f>
@@ -822,7 +867,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B10">
         <f ca="1">_xll.RedisRTDTopicCount()</f>
@@ -831,7 +876,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B11">
         <f ca="1">_xll.RedisRTDSubscriptionCount()</f>
@@ -840,7 +885,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B12">
         <f ca="1">_xll.RedisRTDChannelCount()</f>
@@ -849,7 +894,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B13" t="str">
         <f ca="1">_xll.RedisRTDDefaultHost()</f>
@@ -858,7 +903,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B14">
         <f ca="1">_xll.RedisRTDExcelUpdateInterval()</f>
@@ -867,7 +912,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B15">
         <f ca="1">_xll.RedisRTDRedisUpdateInterval()</f>
@@ -876,7 +921,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B16" t="b">
         <f ca="1">_xll.RedisRTDRealTimeUpdates()</f>

</xml_diff>

<commit_message>
Coalesce real-time updates per topic (CoalesceRealtimeUpdates, default on)
In real-time mode each topic now sends at most one value per ExcelUpdateRateMs
window (the latest value wins) instead of one Excel update per incoming
message; the Excel timer flushes dirty topics in every mode. Set
"CoalesceRealtimeUpdates": false in RedisExcel.json to restore per-message
delivery. The default is the more performant option, per project decision.

Also updated: samples (RedisExcel.json, Readme), AGENTS runtime model,
CHANGELOG (v1.1.4) and the AppConfig defaults test.

Validated: 42 unit tests, smoke tests and the Excel end-to-end suite pass.
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Trabalho\rs\redisexcel\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F837E30E-E852-4F1E-9DAF-FA514E05042E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{74C505F9-D9EA-4227-B08C-1CD3FC5ADA4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5640" yWindow="-28770" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{FF395B52-4190-4BF1-AE53-299997F12B4F}"/>
+    <workbookView xWindow="5640" yWindow="-28770" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{7DCCFD11-588E-476C-99AA-9DD73AD6168A}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -577,7 +577,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{927A6C7C-9621-4CA0-8B6B-51495E5D03BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F6404B3-2E51-47D8-8DC4-93DF1B0E6145}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -782,7 +782,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F3DEB0-CC94-4B2A-A945-A35DD515B1E7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E2A475C-EA32-44E3-87B8-91352767C45F}">
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Polish final audit lows: disconnect defense, sanitizer hardening, E2E checks
- RTD: re-check Disconnected inside the per-topic lock before pushing, so a
  topic disconnected while waiting for the lock is skipped; failed tick pushes
  are now logged outside the lock so a slow log write cannot delay producers.
- E2E sanitizer: use (?s) patterns (multi-line metadata values), sanitize
  docProps/app.xml Company/Manager, and run on the staged copy BEFORE it
  replaces the sample (a failed sanitize leaves the previous sample untouched).
- E2E: regression checks for the RTD argument validation (a missing-key topic
  returns #ERROR without disturbing the host's other topics) and for a
  whitespace-only key; changelog notes them.

Validated: 58 unit tests, smoke, E2E (26s) all pass; sample workbook clean.
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6021AD0C-3095-48A8-BA17-B5813DB399E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{675F28A0-D04B-4C84-A89C-029E764D315D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{74C0D61D-78F1-4ABE-9265-B10751B5643D}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{6A1CB3C3-CA8A-456F-B006-CED773E5E31C}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="68">
   <si>
     <t>RedisExcel UDF tests (host localhost:6379, prefix test.redisexcel)</t>
   </si>
@@ -233,6 +233,15 @@
   </si>
   <si>
     <t>RealTimeUpdates</t>
+  </si>
+  <si>
+    <t>GET missing key</t>
+  </si>
+  <si>
+    <t>GET whitespace key</t>
+  </si>
+  <si>
+    <t>ws_key_value</t>
   </si>
 </sst>
 </file>
@@ -309,6 +318,12 @@
         <tr r="B5" s="2"/>
       </tp>
       <tp t="s">
+        <v>#ERROR: ConnectData: GET requires a key as the second argument</v>
+        <stp/>
+        <stp>GET</stp>
+        <tr r="B20" s="2"/>
+      </tp>
+      <tp t="s">
         <v>ALTA</v>
         <stp/>
         <stp>PSUB</stp>
@@ -331,6 +346,14 @@
         <stp>test.redisexcel.key</stp>
         <stp>localhost:6379</stp>
         <tr r="B4" s="2"/>
+      </tp>
+      <tp t="s">
+        <v>ws_key_value</v>
+        <stp/>
+        <stp>GET</stp>
+        <stp xml:space="preserve"> </stp>
+        <stp>localhost:6379</stp>
+        <tr r="B21" s="2"/>
       </tp>
     </main>
   </volType>
@@ -653,7 +676,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E02B1D6-AE72-45B6-873D-43D0E8D1ED81}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{492AC1C8-B5E6-4FF1-B83F-197889D4D90B}">
   <dimension ref="A1:H37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -873,7 +896,7 @@
       </c>
       <c r="B19">
         <f ca="1">_xll.RedisUDFTTL("test.redisexcel.tmp","localhost:6379")</f>
-        <v>98</v>
+        <v>98.003</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -897,7 +920,7 @@
       </c>
       <c r="B21">
         <f ca="1">_xll.RedisUDFIncr("test.redisexcel.counter","localhost:6379")</f>
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -906,7 +929,7 @@
       </c>
       <c r="B22">
         <f ca="1">_xll.RedisUDFListPushRight("test.redisexcel.list","a","localhost:6379")</f>
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1089,8 +1112,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FA3CE4D-1117-443C-B0CB-C07FCCD8CB51}">
-  <dimension ref="A1:C16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ECDE5F6-AC68-49B5-AE01-DE8FC87A9788}">
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1178,7 +1201,7 @@
       </c>
       <c r="B10">
         <f ca="1">_xll.RedisRTDTopicCount()</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1233,6 +1256,27 @@
       <c r="B16" t="b">
         <f ca="1">_xll.RedisRTDRealTimeUpdates()</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" t="str">
+        <f>RTD("redisrtd",,"GET")</f>
+        <v>#ERROR: ConnectData: GET requires a key as the second argument</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" t="str">
+        <f>RTD("redisrtd",,"GET"," ","localhost:6379")</f>
+        <v>ws_key_value</v>
+      </c>
+      <c r="C21" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final adversarial fixes: batch writer shapes, numeric coercion, unsubscribe guard
- SetKV/SetKVPair/HashSetMultiple validate range shapes before touching Redis
  (row-major flattening, equal cell counts, horizontal 2-row ranges accepted)
  instead of silently writing only part of the data.
- ToInt64Invariant rejects booleans and fractional numbers (TTL and increment
  arguments must be whole numbers).
- RedisUDFChannelUnsubscribe rejects a blank channel instead of reporting
  success for nothing.
- GetMultiple's multipleColumns coerces TRUE/FALSE, 0/1 and text and rejects
  anything else instead of silently meaning FALSE.
- Tests: 90 total (+6) and E2E row 43 (SetKV rejects mismatched counts).

Validated: 90 unit tests, smoke, E2E (22s) all pass.
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4939C1D-B5E5-433A-B26A-A68AEE3AC6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{718E9C97-F3BD-48EA-9D2C-DBF4AC74E041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{9B7465AA-6FDB-4F3D-988B-81C7F7636BDD}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{314ABDF6-4D98-4849-A9C5-078FB1684D1B}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="75">
   <si>
     <t>RedisExcel UDF tests (host localhost:6379, prefix test.redisexcel)</t>
   </si>
@@ -209,6 +209,9 @@
   </si>
   <si>
     <t>GetMultiple 2x2</t>
+  </si>
+  <si>
+    <t>SetKV mismatched</t>
   </si>
   <si>
     <t>RedisExcel RTD tests (host localhost:6379)</t>
@@ -694,8 +697,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{260B408D-23B5-436D-B088-28C0A70F2DB5}">
-  <dimension ref="A1:H42"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9872A662-9EB2-41B4-B0E1-22D68B3BC39D}">
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -914,7 +917,7 @@
       </c>
       <c r="B19">
         <f ca="1">_xll.RedisUDFTTL("test.redisexcel.tmp","localhost:6379")</f>
-        <v>97.991</v>
+        <v>98.015000000000001</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -938,7 +941,7 @@
       </c>
       <c r="B21">
         <f ca="1">_xll.RedisUDFIncr("test.redisexcel.counter","localhost:6379")</f>
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -947,7 +950,7 @@
       </c>
       <c r="B22">
         <f ca="1">_xll.RedisUDFListPushRight("test.redisexcel.list","a","localhost:6379")</f>
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1170,6 +1173,15 @@
       <c r="B42" t="str">
         <f ca="1">INDEX(_xll.RedisUDFGetMultiple($F$2:$G$3,TRUE,"localhost:6379"),2,1)</f>
         <v>linha1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>57</v>
+      </c>
+      <c r="B43" t="str">
+        <f ca="1">_xll.RedisUDFSetKV($F$2:$G$2,$F$3)</f>
+        <v>Error: keys and values must have the same number of cells</v>
       </c>
     </row>
   </sheetData>
@@ -1178,13 +1190,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{570C164C-BACA-45EE-A434-9925DD3C362F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B555F199-EC81-457D-836F-A9521B159827}">
   <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1200,7 +1212,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B4" t="str">
         <f>RTD("redisrtd",,"GET","test.redisexcel.key","localhost:6379")</f>
@@ -1212,7 +1224,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B5" t="str">
         <f>RTD("redisrtd",,"HGET","test.redisexcel.hash","campo1","localhost:6379")</f>
@@ -1224,19 +1236,19 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" t="str">
         <f>RTD("redisrtd",,"HGETALL","test.redisexcel.hash","localhost:6379")</f>
         <v>{"campo1":"valor1"}</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B7" t="str">
         <f>RTD("redisrtd",,"SUB","test.redisexcel.rtd","localhost:6379")</f>
@@ -1245,7 +1257,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B8" t="str">
         <f>RTD("redisrtd",,"PSUB","test.redisexcel.rtd*","localhost:6379")</f>
@@ -1263,7 +1275,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B10">
         <f ca="1">_xll.RedisRTDTopicCount()</f>
@@ -1272,7 +1284,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B11">
         <f ca="1">_xll.RedisRTDSubscriptionCount()</f>
@@ -1281,7 +1293,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B12">
         <f ca="1">_xll.RedisRTDChannelCount()</f>
@@ -1290,7 +1302,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B13" t="str">
         <f ca="1">_xll.RedisRTDDefaultHost()</f>
@@ -1299,7 +1311,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B14">
         <f ca="1">_xll.RedisRTDExcelUpdateInterval()</f>
@@ -1308,7 +1320,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B15">
         <f ca="1">_xll.RedisRTDRedisUpdateInterval()</f>
@@ -1317,7 +1329,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B16" t="b">
         <f ca="1">_xll.RedisRTDRealTimeUpdates()</f>
@@ -1326,7 +1338,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B20" t="str">
         <f>RTD("redisrtd",,"GET")</f>
@@ -1335,14 +1347,14 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B21" t="str">
         <f>RTD("redisrtd",,"GET"," ","localhost:6379")</f>
         <v>ws_key_value</v>
       </c>
       <c r="C21" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ExcelJson guards, E2E/CI and docs for v1.2.7
- ExcelJson: BOM tolerated, MaxDepth 256, oversized matrices rejected before allocation; tests for deep JSON, boolean casing, BOM and the size guard.
- E2E: B12 check, HGETALL {} row, poll-change detection, 2x2 pair layout, PublishIfChanged suppression with forced recalculation.
- CI: release moved to its own job with contents: write scoped to it; v*-rc tags publish as prerelease.
- Docs/changelog: volatile-by-design, sentinels, PublishDedupCacheSize, config read-once; v1.2.7 (unreleased).
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8D2F3AE-08A6-4969-929A-0944F299863E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B4EFD20-9E5E-464A-B939-5F663FD3B8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8971DE97-93A0-48AB-A3A1-2FEF3297C564}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{850A31EE-C1CF-48F5-A90C-C80F2B0686A9}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="81">
   <si>
     <t>RedisExcel UDF tests (host localhost:6379, prefix test.redisexcel)</t>
   </si>
@@ -223,6 +223,12 @@
     <t>Unsubscribe blank channel</t>
   </si>
   <si>
+    <t>HashSetMultiple pairs</t>
+  </si>
+  <si>
+    <t>HashGet pairs</t>
+  </si>
+  <si>
     <t>RedisExcel RTD tests (host localhost:6379)</t>
   </si>
   <si>
@@ -272,6 +278,9 @@
   </si>
   <si>
     <t>ws_key_value</t>
+  </si>
+  <si>
+    <t>HGETALL missing hash</t>
   </si>
 </sst>
 </file>
@@ -348,6 +357,14 @@
         <tr r="B5" s="2"/>
       </tp>
       <tp t="s">
+        <v>{}</v>
+        <stp/>
+        <stp>HGETALL</stp>
+        <stp>test.redisexcel.missinghash</stp>
+        <stp>localhost:6379</stp>
+        <tr r="B22" s="2"/>
+      </tp>
+      <tp t="s">
         <v>#ERROR: ConnectData: GET requires a key as the second argument</v>
         <stp/>
         <stp>GET</stp>
@@ -370,7 +387,7 @@
         <tr r="B7" s="2"/>
       </tp>
       <tp t="s">
-        <v>hello_from_udf</v>
+        <v>hello_v2</v>
         <stp/>
         <stp>GET</stp>
         <stp>test.redisexcel.key</stp>
@@ -378,7 +395,7 @@
         <tr r="B4" s="2"/>
       </tp>
       <tp t="s">
-        <v>ws_key_value</v>
+        <v>(no value)</v>
         <stp/>
         <stp>GET</stp>
         <stp xml:space="preserve"> </stp>
@@ -706,8 +723,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A51F1B98-4C9B-41BD-99C1-A1F6F42668C7}">
-  <dimension ref="A1:H45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C4C6ADD-984A-4084-8E24-C597D6F40A32}">
+  <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -761,7 +778,7 @@
       </c>
       <c r="B5" t="str">
         <f ca="1">_xll.RedisUDFGet("test.redisexcel.key","localhost:6379")</f>
-        <v>hello_from_udf</v>
+        <v>hello_v2</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -926,7 +943,7 @@
       </c>
       <c r="B19">
         <f ca="1">_xll.RedisUDFTTL("test.redisexcel.tmp","localhost:6379")</f>
-        <v>98.196999999999989</v>
+        <v>98.491</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -950,7 +967,7 @@
       </c>
       <c r="B21">
         <f ca="1">_xll.RedisUDFIncr("test.redisexcel.counter","localhost:6379")</f>
-        <v>129</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -959,7 +976,7 @@
       </c>
       <c r="B22">
         <f ca="1">_xll.RedisUDFListPushRight("test.redisexcel.list","a","localhost:6379")</f>
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1212,6 +1229,27 @@
       <c r="B45" t="str">
         <f ca="1">_xll.RedisUDFChannelUnsubscribe("   ")</f>
         <v>Error: a channel is required</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>61</v>
+      </c>
+      <c r="B46" t="str">
+        <f ca="1">_xll.RedisUDFHashSetMultiple("test.redisexcel.pairs",$F$2:$G$3,"localhost:6379")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" t="str">
+        <f ca="1">_xll.RedisUDFHashGet("test.redisexcel.pairs","1","localhost:6379")</f>
+        <v>linha1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1220,13 +1258,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45F33BF0-FFB0-41FB-A58D-35C41A220545}">
-  <dimension ref="A1:C21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E8B336C-6AFB-4024-AF07-FB26C8A403FC}">
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1242,11 +1280,11 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B4" t="str">
         <f>RTD("redisrtd",,"GET","test.redisexcel.key","localhost:6379")</f>
-        <v>hello_from_udf</v>
+        <v>hello_v2</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -1254,7 +1292,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B5" t="str">
         <f>RTD("redisrtd",,"HGET","test.redisexcel.hash","campo1","localhost:6379")</f>
@@ -1266,19 +1304,19 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B6" t="str">
         <f>RTD("redisrtd",,"HGETALL","test.redisexcel.hash","localhost:6379")</f>
         <v>{"campo1":"valor1"}</v>
       </c>
       <c r="C6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B7" t="str">
         <f>RTD("redisrtd",,"SUB","test.redisexcel.rtd","localhost:6379")</f>
@@ -1287,7 +1325,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B8" t="str">
         <f>RTD("redisrtd",,"PSUB","test.redisexcel.rtd*","localhost:6379")</f>
@@ -1300,21 +1338,21 @@
       </c>
       <c r="B9">
         <f ca="1">_xll.RedisRTDConnectionCount()</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B10">
         <f ca="1">_xll.RedisRTDTopicCount()</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B11">
         <f ca="1">_xll.RedisRTDSubscriptionCount()</f>
@@ -1323,7 +1361,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B12">
         <f ca="1">_xll.RedisRTDChannelCount()</f>
@@ -1332,7 +1370,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B13" t="str">
         <f ca="1">_xll.RedisRTDDefaultHost()</f>
@@ -1341,7 +1379,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B14">
         <f ca="1">_xll.RedisRTDExcelUpdateInterval()</f>
@@ -1350,7 +1388,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B15">
         <f ca="1">_xll.RedisRTDRedisUpdateInterval()</f>
@@ -1359,7 +1397,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B16" t="b">
         <f ca="1">_xll.RedisRTDRealTimeUpdates()</f>
@@ -1368,7 +1406,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B20" t="str">
         <f>RTD("redisrtd",,"GET")</f>
@@ -1377,14 +1415,23 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B21" t="str">
         <f>RTD("redisrtd",,"GET"," ","localhost:6379")</f>
-        <v>ws_key_value</v>
+        <v>(no value)</v>
       </c>
       <c r="C21" t="s">
-        <v>77</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" t="str">
+        <f>RTD("redisrtd",,"HGETALL","test.redisexcel.missinghash","localhost:6379")</f>
+        <v>{}</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ExcelJson BOM trim, docs, E2E poll-change retry
- ExcelJson: leading whitespace before a BOM is tolerated (whitespace/BOM-only input maps to the fill).
- E2E: the polled-GET check re-issues the SET until the RTD cell shows the new value - the volatile Set row rewrites the key on the recalculation triggered around the first push, which made the check racy by design.
- Docs: volatile-by-design wording (JSON conversions excepted), per-pool live counters, join-based marker clearing, ChannelLatest best-effort note, retry backoff, changelog corrections.
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B4EFD20-9E5E-464A-B939-5F663FD3B8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D3DB787A-BCEF-480C-B331-4F59707A148A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{850A31EE-C1CF-48F5-A90C-C80F2B0686A9}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{E1482016-A736-4F64-B836-B1BB5E789429}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -723,7 +723,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C4C6ADD-984A-4084-8E24-C597D6F40A32}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9859F707-378E-40EB-B1D7-FAB277FDDEE8}">
   <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -778,7 +778,7 @@
       </c>
       <c r="B5" t="str">
         <f ca="1">_xll.RedisUDFGet("test.redisexcel.key","localhost:6379")</f>
-        <v>hello_v2</v>
+        <v>hello_from_udf</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -943,7 +943,7 @@
       </c>
       <c r="B19">
         <f ca="1">_xll.RedisUDFTTL("test.redisexcel.tmp","localhost:6379")</f>
-        <v>98.491</v>
+        <v>98.001999999999995</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -967,7 +967,7 @@
       </c>
       <c r="B21">
         <f ca="1">_xll.RedisUDFIncr("test.redisexcel.counter","localhost:6379")</f>
-        <v>143</v>
+        <v>446</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -976,7 +976,7 @@
       </c>
       <c r="B22">
         <f ca="1">_xll.RedisUDFListPushRight("test.redisexcel.list","a","localhost:6379")</f>
-        <v>140</v>
+        <v>437</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1258,7 +1258,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E8B336C-6AFB-4024-AF07-FB26C8A403FC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A94FE498-E965-460B-A1EE-4BF0B2F32D36}">
   <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B9">
         <f ca="1">_xll.RedisRTDConnectionCount()</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Refresh the E2E sample workbook
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA4C3169-0C45-40AF-AC61-2C4CEC847B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E20FEF76-C3D0-4640-9A4A-0275629EBED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{2DA2DB09-C080-4006-B58F-5BF1BAA66049}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{6FDCA6AA-6EFF-4BB1-B64B-400EC0A4D9BC}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -353,6 +353,58 @@
         <stp>localhost:6379</stp>
         <tr r="B6" s="2"/>
       </tp>
+    </main>
+    <main first="rtdsrv_43a5ede2991d42c0b8004436e2e2364b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>682e6eb1-5329-4ed1-929b-5742b20c9f44</stp>
+        <tr r="B45" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_43a5ede2991d42c0b8004436e2e2364b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>524252c7-c97d-4421-a1e4-bd1fa24a9f9e</stp>
+        <tr r="B31" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_43a5ede2991d42c0b8004436e2e2364b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>9145b6e4-d0e6-4c1b-997f-ac25936d1c9b</stp>
+        <tr r="B21" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>c9156aca-36cc-40a2-8f2e-f25640b34c3b</stp>
+        <tr r="B10" s="1"/>
+      </tp>
+    </main>
+    <main first="rtdsrv_43a5ede2991d42c0b8004436e2e2364b">
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>f0ba7a59-f950-43cb-8584-31e280b7ddff</stp>
+        <tr r="B37" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>626cdfdd-9a18-4399-beef-997f0920f927</stp>
+        <tr r="B35" s="1"/>
+      </tp>
+      <tp>
+        <v>1</v>
+        <stp/>
+        <stp>7078a8ae-5da0-4240-bf50-804dd52fd064</stp>
+        <tr r="B43" s="1"/>
+      </tp>
+    </main>
+    <main first="redisrtd">
       <tp t="s">
         <v>valor1</v>
         <stp/>
@@ -370,6 +422,8 @@
         <stp>localhost:6379</stp>
         <tr r="B22" s="2"/>
       </tp>
+    </main>
+    <main first="redisrtd">
       <tp t="s">
         <v>#ERROR: ConnectData: GET requires a key as the second argument</v>
         <stp/>
@@ -729,7 +783,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB053C72-EB91-4742-8D74-6612A274FAB8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B27F2B0-BB9E-40C4-81FF-A71251313A1F}">
   <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -772,7 +826,7 @@
       </c>
       <c r="B4" t="str">
         <f ca="1">_xll.RedisUDFSet("test.redisexcel.key","hello_from_udf","localhost:6379")</f>
-        <v>OK</v>
+        <v>OK FireForget</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -784,7 +838,7 @@
       </c>
       <c r="B5" t="str">
         <f ca="1">_xll.RedisUDFGet("test.redisexcel.key","localhost:6379")</f>
-        <v>hello_v2</v>
+        <v>hello_from_udf</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -820,7 +874,7 @@
       </c>
       <c r="B8" t="str">
         <f ca="1">_xll.RedisUDFSetJSON("test.redisexcel.json",$F$2:$G$3,"localhost:6379")</f>
-        <v>OK</v>
+        <v>OK FireForget</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
@@ -842,9 +896,9 @@
       <c r="A10" t="s">
         <v>14</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B10" t="e">
         <f ca="1">_xll.RedisUDFHashSet("test.redisexcel.hash","campo1","valor1","localhost:6379")</f>
-        <v>OK</v>
+        <v>#N/A</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
@@ -868,7 +922,7 @@
       </c>
       <c r="B12" t="str">
         <f ca="1">_xll.RedisUDFChannelPublish("test.redisexcel.channel","ola_mundo","localhost:6379")</f>
-        <v>1 readers(s)</v>
+        <v>OK FireForget</v>
       </c>
       <c r="C12" t="s">
         <v>18</v>
@@ -937,7 +991,7 @@
       </c>
       <c r="B18" t="str">
         <f ca="1">_xll.RedisUDFSetEx("test.redisexcel.tmp","x","100","localhost:6379")</f>
-        <v>OK</v>
+        <v>OK FireForget</v>
       </c>
       <c r="C18" t="s">
         <v>7</v>
@@ -949,7 +1003,7 @@
       </c>
       <c r="B19">
         <f ca="1">_xll.RedisUDFTTL("test.redisexcel.tmp","localhost:6379")</f>
-        <v>98.546999999999997</v>
+        <v>99.673999999999992</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -971,18 +1025,18 @@
       <c r="A21" t="s">
         <v>27</v>
       </c>
-      <c r="B21">
+      <c r="B21" t="e">
         <f ca="1">_xll.RedisUDFIncr("test.redisexcel.counter","localhost:6379")</f>
-        <v>150</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>28</v>
       </c>
-      <c r="B22">
+      <c r="B22" t="str">
         <f ca="1">_xll.RedisUDFListPushRight("test.redisexcel.list","a","localhost:6379")</f>
-        <v>147</v>
+        <v>OK FireForget</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1024,7 +1078,7 @@
       </c>
       <c r="B26" t="str">
         <f ca="1">_xll.RedisUDFSet("test.redisexcel.locale",$H$2,"localhost:6379")</f>
-        <v>OK</v>
+        <v>OK FireForget</v>
       </c>
       <c r="C26" t="s">
         <v>7</v>
@@ -1048,7 +1102,7 @@
       </c>
       <c r="B28" t="str">
         <f ca="1">_xll.RedisUDFSet($H$2,"dec-key","localhost:6379")</f>
-        <v>OK</v>
+        <v>OK FireForget</v>
       </c>
       <c r="C28" t="s">
         <v>7</v>
@@ -1082,9 +1136,9 @@
       <c r="A31" t="s">
         <v>40</v>
       </c>
-      <c r="B31">
+      <c r="B31" t="e">
         <f ca="1">_xll.RedisUDFSetRemove("test.redisexcel.set","missing","localhost:6379")</f>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -1130,9 +1184,9 @@
       <c r="A35" t="s">
         <v>47</v>
       </c>
-      <c r="B35" t="str">
+      <c r="B35" t="e">
         <f ca="1">IF(_xll.RedisUDFListPopRight("test.redisexcel.emptylist","localhost:6379")="","empty","not empty")</f>
-        <v>empty</v>
+        <v>#N/A</v>
       </c>
       <c r="C35" t="s">
         <v>48</v>
@@ -1154,9 +1208,9 @@
       <c r="A37" t="s">
         <v>50</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B37" t="e">
         <f ca="1">_xll.RedisUDFRename("test.redisexcel.missingrename","test.redisexcel.renamed","localhost:6379")</f>
-        <v>Error: ERR no such key</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1211,9 +1265,9 @@
       <c r="A43" t="s">
         <v>57</v>
       </c>
-      <c r="B43" t="str">
+      <c r="B43" t="e">
         <f ca="1">_xll.RedisUDFSetKV($F$2:$G$2,$F$3)</f>
-        <v>Error: keys and values must have the same number of cells</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1232,9 +1286,9 @@
       <c r="A45" t="s">
         <v>60</v>
       </c>
-      <c r="B45" t="str">
+      <c r="B45" t="e">
         <f ca="1">_xll.RedisUDFChannelUnsubscribe("   ")</f>
-        <v>Error: a channel is required</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1243,7 +1297,7 @@
       </c>
       <c r="B46" t="str">
         <f ca="1">_xll.RedisUDFHashSetMultiple("test.redisexcel.pairs",$F$2:$G$3,"localhost:6379")</f>
-        <v>OK</v>
+        <v>OK FireForget</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1264,7 +1318,7 @@
       </c>
       <c r="B48" t="str">
         <f>_xll.RedisUDFSetNonVolatile("test.redisexcel.nvkey","v1","localhost:6379")</f>
-        <v>OK</v>
+        <v>OK FireForget</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -1282,7 +1336,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAE65069-E721-431C-A289-74E6CD38CC70}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14363D7F-8E75-488A-BC13-5862E65F4280}">
   <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>

<commit_message>
﻿Docs: complete the v1.6.0 changelog (installer languages, security, fixes)
The release/CHANGELOG audit found the v1.6.0 section omitted several
user-visible changes: the installer's 10 languages, the installed-tooling
improvements (Validate-Config verdict parity + the truncated-password warning),
the credential-masking hardening and the installer/reload fixes made during the
audit rounds. Added Added/Security/Fixed sections (the HA bullet moved into
Added, no duplicate).
</commit_message>
<xml_diff>
--- a/test/RedisExcel.Test.xlsx
+++ b/test/RedisExcel.Test.xlsx
@@ -6,9 +6,9 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23164F3E-5F08-4447-BA01-7AF4E983589B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F81AE0FE-188B-47D1-AD87-A4FE40B876D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{E849E415-158E-4338-9A3C-02BBBAFB98FB}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{1B554EA8-6FB7-40C7-A689-1A251DE17F15}"/>
   </bookViews>
   <sheets>
     <sheet name="UDF" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="85">
   <si>
     <t>RedisExcel UDF tests (host localhost:6379, prefix test.redisexcel)</t>
   </si>
@@ -94,7 +94,7 @@
     <t>ChannelPublish</t>
   </si>
   <si>
-    <t>1 readers(s)</t>
+    <t>1 reader</t>
   </si>
   <si>
     <t>ChannelLatest</t>
@@ -227,6 +227,12 @@
   </si>
   <si>
     <t>HashGet pairs</t>
+  </si>
+  <si>
+    <t>CheckConfigFile</t>
+  </si>
+  <si>
+    <t>JsonSchemaContents length</t>
   </si>
   <si>
     <t>RedisExcel RTD tests (host localhost:6379)</t>
@@ -414,7 +420,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -729,8 +735,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD689C96-BC85-4E21-B81C-21AD42D772BE}">
-  <dimension ref="A1:H49"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEBB5BB5-4203-4FB2-A704-132E090E4B3B}">
+  <dimension ref="A1:H56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -772,7 +778,7 @@
       </c>
       <c r="B4" t="str">
         <f ca="1">_xll.RedisUDFSet("test.redisexcel.key","hello_from_udf","localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -820,7 +826,7 @@
       </c>
       <c r="B8" t="str">
         <f ca="1">_xll.RedisUDFSetJSON("test.redisexcel.json",$F$2:$G$3,"localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
@@ -844,7 +850,7 @@
       </c>
       <c r="B10" t="str">
         <f ca="1">_xll.RedisUDFHashSet("test.redisexcel.hash","campo1","valor1","localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
@@ -868,7 +874,7 @@
       </c>
       <c r="B12" t="str">
         <f ca="1">_xll.RedisUDFChannelPublish("test.redisexcel.channel","ola_mundo","localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
       <c r="C12" t="s">
         <v>18</v>
@@ -937,7 +943,7 @@
       </c>
       <c r="B18" t="str">
         <f ca="1">_xll.RedisUDFSetEx("test.redisexcel.tmp","x","100","localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
       <c r="C18" t="s">
         <v>7</v>
@@ -949,7 +955,7 @@
       </c>
       <c r="B19">
         <f ca="1">_xll.RedisUDFTTL("test.redisexcel.tmp","localhost:6379")</f>
-        <v>98.507999999999996</v>
+        <v>98.575999999999993</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -959,9 +965,9 @@
       <c r="A20" t="s">
         <v>26</v>
       </c>
-      <c r="B20">
+      <c r="B20" t="str">
         <f ca="1">_xll.RedisUDFDel("test.redisexcel.neverexists","localhost:6379")</f>
-        <v>0</v>
+        <v>OK (fire and forget: all)</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -971,9 +977,9 @@
       <c r="A21" t="s">
         <v>27</v>
       </c>
-      <c r="B21">
+      <c r="B21" t="str">
         <f ca="1">_xll.RedisUDFIncr("test.redisexcel.counter","localhost:6379")</f>
-        <v>239</v>
+        <v>OK (fire and forget: all)</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -982,7 +988,7 @@
       </c>
       <c r="B22" t="str">
         <f ca="1">_xll.RedisUDFListPushRight("test.redisexcel.list","a","localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1001,9 +1007,9 @@
       <c r="A24" t="s">
         <v>31</v>
       </c>
-      <c r="B24">
+      <c r="B24" t="str">
         <f ca="1">_xll.RedisUDFSetAdd("test.redisexcel.set","x","localhost:6379")</f>
-        <v>0</v>
+        <v>OK (fire and forget: all)</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1024,7 +1030,7 @@
       </c>
       <c r="B26" t="str">
         <f ca="1">_xll.RedisUDFSet("test.redisexcel.locale",$H$2,"localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
       <c r="C26" t="s">
         <v>7</v>
@@ -1048,7 +1054,7 @@
       </c>
       <c r="B28" t="str">
         <f ca="1">_xll.RedisUDFSet($H$2,"dec-key","localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
       <c r="C28" t="s">
         <v>7</v>
@@ -1070,9 +1076,9 @@
       <c r="A30" t="s">
         <v>39</v>
       </c>
-      <c r="B30">
+      <c r="B30" t="str">
         <f ca="1">_xll.RedisUDFHashDel("test.redisexcel.hash","missing","localhost:6379")</f>
-        <v>0</v>
+        <v>OK (fire and forget: all)</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -1082,9 +1088,9 @@
       <c r="A31" t="s">
         <v>40</v>
       </c>
-      <c r="B31">
+      <c r="B31" t="str">
         <f ca="1">_xll.RedisUDFSetRemove("test.redisexcel.set","missing","localhost:6379")</f>
-        <v>0</v>
+        <v>OK (fire and forget: all)</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -1132,7 +1138,7 @@
       </c>
       <c r="B35" t="str">
         <f ca="1">IF(_xll.RedisUDFListPopRight("test.redisexcel.emptylist","localhost:6379")="","empty","not empty")</f>
-        <v>empty</v>
+        <v>not empty</v>
       </c>
       <c r="C35" t="s">
         <v>48</v>
@@ -1144,7 +1150,7 @@
       </c>
       <c r="B36" t="str">
         <f ca="1">IF(_xll.RedisUDFListPopLeft("test.redisexcel.emptylist","localhost:6379")="","empty","not empty")</f>
-        <v>empty</v>
+        <v>not empty</v>
       </c>
       <c r="C36" t="s">
         <v>48</v>
@@ -1156,7 +1162,7 @@
       </c>
       <c r="B37" t="str">
         <f ca="1">_xll.RedisUDFRename("test.redisexcel.missingrename","test.redisexcel.renamed","localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1243,7 +1249,7 @@
       </c>
       <c r="B46" t="str">
         <f ca="1">_xll.RedisUDFHashSetMultiple("test.redisexcel.pairs",$F$2:$G$3,"localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1260,20 +1266,38 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B48" t="str">
         <f>_xll.RedisUDFSetNonVolatile("test.redisexcel.nvkey","v1","localhost:6379")</f>
-        <v>OK FireForget</v>
+        <v>OK (fire and forget)</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>82</v>
-      </c>
-      <c r="B49">
+        <v>84</v>
+      </c>
+      <c r="B49" t="str">
         <f>_xll.RedisUDFIncrNonVolatile("test.redisexcel.nvcounter","localhost:6379")</f>
-        <v>1</v>
+        <v>OK (fire and forget: all)</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>63</v>
+      </c>
+      <c r="B55" t="str">
+        <f ca="1">_xll.RedisCheckConfigFile()</f>
+        <v>OK (C:\Users\rober\RedisExcel.json)</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>64</v>
+      </c>
+      <c r="B56">
+        <f ca="1">LEN(_xll.RedisJsonSchemaContents())</f>
+        <v>4189</v>
       </c>
     </row>
   </sheetData>
@@ -1282,13 +1306,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38098415-6AA4-472C-B1C4-B7E86F40DCFA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9562012E-06F5-42DF-9D9D-3BC23F20EB3A}">
   <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1304,7 +1328,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B4" t="str">
         <f>RTD("redisrtd",,"GET","test.redisexcel.key","localhost:6379")</f>
@@ -1316,7 +1340,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B5" t="str">
         <f>RTD("redisrtd",,"HGET","test.redisexcel.hash","campo1","localhost:6379")</f>
@@ -1328,19 +1352,19 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B6" t="str">
         <f>RTD("redisrtd",,"HGETALL","test.redisexcel.hash","localhost:6379")</f>
         <v>{"campo1":"valor1"}</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B7" t="str">
         <f>RTD("redisrtd",,"SUB","test.redisexcel.rtd","localhost:6379")</f>
@@ -1349,7 +1373,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B8" t="str">
         <f>RTD("redisrtd",,"PSUB","test.redisexcel.rtd*","localhost:6379")</f>
@@ -1367,7 +1391,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B10">
         <f ca="1">_xll.RedisRTDTopicCount()</f>
@@ -1376,7 +1400,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B11">
         <f ca="1">_xll.RedisRTDSubscriptionCount()</f>
@@ -1385,7 +1409,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12">
         <f ca="1">_xll.RedisRTDChannelCount()</f>
@@ -1394,16 +1418,16 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B13" t="str">
         <f ca="1">_xll.RedisRTDDefaultHost()</f>
-        <v>localhost:6379,password=,defaultDatabase=0,ssl=False,abortConnect=False</v>
+        <v>localhost:6379,password=****,defaultDatabase=0,ssl=False,abortConnect=False</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B14">
         <f ca="1">_xll.RedisRTDExcelUpdateInterval()</f>
@@ -1412,7 +1436,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B15">
         <f ca="1">_xll.RedisRTDRedisUpdateInterval()</f>
@@ -1421,7 +1445,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" t="b">
         <f ca="1">_xll.RedisRTDRealTimeUpdates()</f>
@@ -1430,7 +1454,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B20" t="str">
         <f>RTD("redisrtd",,"GET")</f>
@@ -1439,19 +1463,19 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B21" t="str">
         <f>RTD("redisrtd",,"GET"," ","localhost:6379")</f>
         <v>(no value)</v>
       </c>
       <c r="C21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B22" t="str">
         <f>RTD("redisrtd",,"HGETALL","test.redisexcel.missinghash","localhost:6379")</f>

</xml_diff>